<commit_message>
Se cambió el formato de los datos
</commit_message>
<xml_diff>
--- a/datos/Datosrotativo1.xlsx
+++ b/datos/Datosrotativo1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7815"/>
+    <workbookView windowWidth="20490" windowHeight="7815" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -16,15 +16,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
   <si>
-    <t>Presion por distancia (20cm)</t>
+    <t>Presion por distancia (20cm) [m*Torr]</t>
   </si>
   <si>
     <t>Voltaje [V]</t>
-  </si>
-  <si>
-    <t>m*Torr</t>
   </si>
   <si>
     <t>9-agosto-1ra corrida</t>
@@ -976,10 +973,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="28.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="37.5714285714286" customWidth="1"/>
     <col min="2" max="2" width="11.2857142857143" customWidth="1"/>
     <col min="3" max="3" width="8.56190476190476" customWidth="1"/>
     <col min="4" max="4" width="10.2" customWidth="1"/>
@@ -999,62 +996,65 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>3</v>
+    <row r="3" spans="1:2">
+      <c r="A3">
+        <v>0.00108</v>
+      </c>
+      <c r="B3">
+        <v>3150</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4">
-        <v>0.00108</v>
+        <v>0.0013</v>
       </c>
       <c r="B4">
-        <v>3150</v>
+        <v>840</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5">
-        <v>0.0013</v>
+        <v>0.00148</v>
       </c>
       <c r="B5">
-        <v>840</v>
+        <v>520</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
-        <v>0.00148</v>
+        <v>0.00172</v>
       </c>
       <c r="B6">
-        <v>520</v>
+        <v>450</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>0.00172</v>
+        <v>0.00178</v>
       </c>
       <c r="B7">
-        <v>450</v>
+        <v>413</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>0.00178</v>
+        <v>0.0019</v>
       </c>
       <c r="B8">
-        <v>413</v>
+        <v>380</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9">
-        <v>0.0019</v>
+        <v>0.002</v>
       </c>
       <c r="B9">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10">
-        <v>0.002</v>
+        <v>0.0036</v>
       </c>
       <c r="B10">
         <v>379</v>
@@ -1062,81 +1062,73 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11">
-        <v>0.0036</v>
+        <v>0.0042</v>
       </c>
       <c r="B11">
-        <v>379</v>
+        <v>382</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12">
-        <v>0.0042</v>
+        <v>0.0052</v>
       </c>
       <c r="B12">
-        <v>382</v>
+        <v>410</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13">
-        <v>0.0052</v>
+        <v>0.0066</v>
       </c>
       <c r="B13">
-        <v>410</v>
+        <v>469</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14">
-        <v>0.0066</v>
+        <v>0.007</v>
       </c>
       <c r="B14">
-        <v>469</v>
+        <v>472</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
       <c r="B15">
-        <v>472</v>
+        <v>502</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16">
-        <v>0.008</v>
+        <v>0.0122</v>
       </c>
       <c r="B16">
-        <v>502</v>
+        <v>586</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17">
-        <v>0.0122</v>
+        <v>0.0138</v>
       </c>
       <c r="B17">
-        <v>586</v>
+        <v>615</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18">
-        <v>0.0138</v>
+        <v>0.0172</v>
       </c>
       <c r="B18">
-        <v>615</v>
+        <v>678</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19">
-        <v>0.0172</v>
+        <v>0.0198</v>
       </c>
       <c r="B19">
-        <v>678</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20">
-        <v>0.0198</v>
-      </c>
-      <c r="B20">
         <v>702</v>
       </c>
     </row>
@@ -1149,10 +1141,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="28.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="37.5714285714286" customWidth="1"/>
     <col min="2" max="2" width="11.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1166,83 +1158,85 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1"/>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1"/>
+      <c r="A3" s="1">
+        <v>0.00106</v>
+      </c>
+      <c r="B3" s="1">
+        <v>3080</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1">
-        <v>0.00106</v>
+        <v>0.00118</v>
       </c>
       <c r="B4" s="1">
-        <v>3080</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1">
-        <v>0.00118</v>
+        <v>0.00142</v>
       </c>
       <c r="B5" s="1">
-        <v>1300</v>
+        <v>630</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1">
-        <v>0.00142</v>
+        <v>0.00168</v>
       </c>
       <c r="B6" s="1">
-        <v>630</v>
+        <v>520</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1">
-        <v>0.00168</v>
+        <v>0.00184</v>
       </c>
       <c r="B7" s="1">
-        <v>520</v>
+        <v>450</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1">
-        <v>0.00184</v>
+        <v>0.002</v>
       </c>
       <c r="B8" s="1">
-        <v>450</v>
+        <v>400</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1">
-        <v>0.002</v>
+        <v>0.0028</v>
       </c>
       <c r="B9" s="1">
-        <v>400</v>
+        <v>490</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1">
-        <v>0.0028</v>
+        <v>0.0024</v>
       </c>
       <c r="B10" s="1">
-        <v>490</v>
+        <v>410</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1">
-        <v>0.0024</v>
+        <v>0.003</v>
       </c>
       <c r="B11" s="1">
-        <v>410</v>
+        <v>400</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="1">
-        <v>0.003</v>
+        <v>0.0032</v>
       </c>
       <c r="B12" s="1">
         <v>400</v>
@@ -1250,10 +1244,10 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1">
-        <v>0.0032</v>
+        <v>0.003</v>
       </c>
       <c r="B13" s="1">
-        <v>400</v>
+        <v>390</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -1261,86 +1255,78 @@
         <v>0.003</v>
       </c>
       <c r="B14" s="1">
-        <v>390</v>
+        <v>400</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1">
-        <v>0.003</v>
+        <v>0.0044</v>
       </c>
       <c r="B15" s="1">
-        <v>400</v>
+        <v>420</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1">
-        <v>0.0044</v>
+        <v>0.0058</v>
       </c>
       <c r="B16" s="1">
-        <v>420</v>
+        <v>431</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1">
-        <v>0.0058</v>
+        <v>0.0066</v>
       </c>
       <c r="B17" s="1">
-        <v>431</v>
+        <v>435</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1">
-        <v>0.0066</v>
+        <v>0.0086</v>
       </c>
       <c r="B18" s="1">
-        <v>435</v>
+        <v>490</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1">
-        <v>0.0086</v>
+        <v>0.0096</v>
       </c>
       <c r="B19" s="1">
-        <v>490</v>
+        <v>500</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1">
-        <v>0.0096</v>
+        <v>0.0116</v>
       </c>
       <c r="B20" s="1">
-        <v>500</v>
+        <v>552</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1">
-        <v>0.0116</v>
+        <v>0.0148</v>
       </c>
       <c r="B21" s="1">
-        <v>552</v>
+        <v>640</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1">
-        <v>0.0148</v>
+        <v>0.0166</v>
       </c>
       <c r="B22" s="1">
-        <v>640</v>
+        <v>652</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="1">
-        <v>0.0166</v>
+        <v>0.019</v>
       </c>
       <c r="B23" s="1">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" s="1">
-        <v>0.019</v>
-      </c>
-      <c r="B24" s="1">
         <v>697</v>
       </c>
     </row>
@@ -1353,10 +1339,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="28.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="37.5714285714286" customWidth="1"/>
     <col min="2" max="2" width="11.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1370,78 +1356,80 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1"/>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1"/>
+      <c r="A3" s="1">
+        <v>0.00102</v>
+      </c>
+      <c r="B3" s="1">
+        <v>3038</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1">
-        <v>0.00102</v>
+        <v>0.00116</v>
       </c>
       <c r="B4" s="1">
-        <v>3038</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1">
-        <v>0.00116</v>
+        <v>0.00142</v>
       </c>
       <c r="B5" s="1">
-        <v>1197</v>
+        <v>476</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1">
-        <v>0.00142</v>
+        <v>0.00154</v>
       </c>
       <c r="B6" s="1">
-        <v>476</v>
+        <v>513</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1">
-        <v>0.00154</v>
+        <v>0.00168</v>
       </c>
       <c r="B7" s="1">
-        <v>513</v>
+        <v>453</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1">
-        <v>0.00168</v>
+        <v>0.00186</v>
       </c>
       <c r="B8" s="1">
-        <v>453</v>
+        <v>412</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1">
-        <v>0.00186</v>
+        <v>0.002</v>
       </c>
       <c r="B9" s="1">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1">
-        <v>0.002</v>
+        <v>0.0022</v>
       </c>
       <c r="B10" s="1">
-        <v>413</v>
+        <v>390</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1">
-        <v>0.0022</v>
+        <v>0.0028</v>
       </c>
       <c r="B11" s="1">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -1449,94 +1437,86 @@
         <v>0.0028</v>
       </c>
       <c r="B12" s="1">
-        <v>392</v>
+        <v>340</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="1">
-        <v>0.0028</v>
+        <v>0.0044</v>
       </c>
       <c r="B13" s="1">
-        <v>340</v>
+        <v>420</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="1">
-        <v>0.0044</v>
+        <v>0.0046</v>
       </c>
       <c r="B14" s="1">
-        <v>420</v>
+        <v>424</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="1">
-        <v>0.0046</v>
+        <v>0.005</v>
       </c>
       <c r="B15" s="1">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="1">
-        <v>0.005</v>
+        <v>0.0066</v>
       </c>
       <c r="B16" s="1">
-        <v>425</v>
+        <v>466</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="1">
-        <v>0.0066</v>
+        <v>0.0088</v>
       </c>
       <c r="B17" s="1">
-        <v>466</v>
+        <v>487</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="1">
-        <v>0.0088</v>
+        <v>0.0102</v>
       </c>
       <c r="B18" s="1">
-        <v>487</v>
+        <v>532</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="1">
-        <v>0.0102</v>
+        <v>0.0116</v>
       </c>
       <c r="B19" s="1">
-        <v>532</v>
+        <v>557</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="1">
-        <v>0.0116</v>
+        <v>0.013</v>
       </c>
       <c r="B20" s="1">
-        <v>557</v>
+        <v>579</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="1">
-        <v>0.013</v>
+        <v>0.0152</v>
       </c>
       <c r="B21" s="1">
-        <v>579</v>
+        <v>631</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="1">
-        <v>0.0152</v>
+        <v>0.0174</v>
       </c>
       <c r="B22" s="1">
-        <v>631</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="1">
-        <v>0.0174</v>
-      </c>
-      <c r="B23" s="1">
         <v>694</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Se agregaron datos para d=10 en el aire
</commit_message>
<xml_diff>
--- a/datos/Datosrotativo1.xlsx
+++ b/datos/Datosrotativo1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7815" activeTab="1"/>
+    <workbookView windowWidth="20490" windowHeight="7815"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -38,12 +38,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -52,22 +52,47 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -75,68 +100,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -181,6 +145,27 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
@@ -189,6 +174,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Calibri"/>
@@ -197,7 +190,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -212,13 +205,109 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -230,19 +319,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -254,145 +361,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -411,17 +404,6 @@
       <top/>
       <bottom style="medium">
         <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -480,6 +462,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="double">
         <color rgb="FF3F3F3F"/>
       </left>
@@ -497,157 +488,159 @@
     <border>
       <left/>
       <right/>
-      <top/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
       <bottom style="double">
-        <color rgb="FFFF8001"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -978,9 +971,11 @@
   <cols>
     <col min="1" max="1" width="37.5714285714286" customWidth="1"/>
     <col min="2" max="2" width="11.2857142857143" customWidth="1"/>
-    <col min="3" max="3" width="8.56190476190476" customWidth="1"/>
-    <col min="4" max="4" width="10.2" customWidth="1"/>
-    <col min="5" max="6" width="35.1428571428571" customWidth="1"/>
+    <col min="3" max="4" width="9.2" customWidth="1"/>
+    <col min="5" max="5" width="9.51428571428571" customWidth="1"/>
+    <col min="6" max="6" width="9.37142857142857" customWidth="1"/>
+    <col min="7" max="7" width="10.3238095238095" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>